<commit_message>
feat: incorpora PDV real (10.100 em 2026 + 3k/ano) na projeção e corrige bug dos gráficos
</commit_message>
<xml_diff>
--- a/dados/pessoal_tratado.xlsx
+++ b/dados/pessoal_tratado.xlsx
@@ -1318,7 +1318,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1344,10 +1344,15 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>PDV_Voluntario</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Total_Saidas</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Efetivo_Projetado</t>
         </is>
@@ -1367,10 +1372,13 @@
         <v>330</v>
       </c>
       <c r="E2" t="n">
-        <v>1705</v>
+        <v>10100</v>
       </c>
       <c r="F2" t="n">
-        <v>86384</v>
+        <v>11805</v>
+      </c>
+      <c r="G2" t="n">
+        <v>76284</v>
       </c>
     </row>
     <row r="3">
@@ -1387,10 +1395,13 @@
         <v>352</v>
       </c>
       <c r="E3" t="n">
-        <v>1815</v>
+        <v>3000</v>
       </c>
       <c r="F3" t="n">
-        <v>84569</v>
+        <v>4815</v>
+      </c>
+      <c r="G3" t="n">
+        <v>71469</v>
       </c>
     </row>
     <row r="4">
@@ -1407,10 +1418,13 @@
         <v>385</v>
       </c>
       <c r="E4" t="n">
-        <v>1970</v>
+        <v>3000</v>
       </c>
       <c r="F4" t="n">
-        <v>82599</v>
+        <v>4970</v>
+      </c>
+      <c r="G4" t="n">
+        <v>66499</v>
       </c>
     </row>
     <row r="5">
@@ -1427,10 +1441,13 @@
         <v>418</v>
       </c>
       <c r="E5" t="n">
-        <v>2058</v>
+        <v>3000</v>
       </c>
       <c r="F5" t="n">
-        <v>80541</v>
+        <v>5058</v>
+      </c>
+      <c r="G5" t="n">
+        <v>61441</v>
       </c>
     </row>
     <row r="6">
@@ -1447,10 +1464,13 @@
         <v>440</v>
       </c>
       <c r="E6" t="n">
-        <v>2201</v>
+        <v>3000</v>
       </c>
       <c r="F6" t="n">
-        <v>78340</v>
+        <v>5201</v>
+      </c>
+      <c r="G6" t="n">
+        <v>56240</v>
       </c>
     </row>
     <row r="7">
@@ -1467,10 +1487,13 @@
         <v>462</v>
       </c>
       <c r="E7" t="n">
-        <v>2256</v>
+        <v>3000</v>
       </c>
       <c r="F7" t="n">
-        <v>76084</v>
+        <v>5256</v>
+      </c>
+      <c r="G7" t="n">
+        <v>50984</v>
       </c>
     </row>
     <row r="8">
@@ -1487,10 +1510,13 @@
         <v>495</v>
       </c>
       <c r="E8" t="n">
-        <v>2300</v>
+        <v>3000</v>
       </c>
       <c r="F8" t="n">
-        <v>73784</v>
+        <v>5300</v>
+      </c>
+      <c r="G8" t="n">
+        <v>45684</v>
       </c>
     </row>
     <row r="9">
@@ -1507,10 +1533,13 @@
         <v>517</v>
       </c>
       <c r="E9" t="n">
-        <v>2344</v>
+        <v>3000</v>
       </c>
       <c r="F9" t="n">
-        <v>71440</v>
+        <v>5344</v>
+      </c>
+      <c r="G9" t="n">
+        <v>40340</v>
       </c>
     </row>
     <row r="10">
@@ -1527,10 +1556,13 @@
         <v>539</v>
       </c>
       <c r="E10" t="n">
-        <v>2311</v>
+        <v>3000</v>
       </c>
       <c r="F10" t="n">
-        <v>69129</v>
+        <v>5311</v>
+      </c>
+      <c r="G10" t="n">
+        <v>35029</v>
       </c>
     </row>
     <row r="11">
@@ -1547,10 +1579,13 @@
         <v>550</v>
       </c>
       <c r="E11" t="n">
-        <v>2212</v>
+        <v>3000</v>
       </c>
       <c r="F11" t="n">
-        <v>66917</v>
+        <v>5212</v>
+      </c>
+      <c r="G11" t="n">
+        <v>29817</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: implementa projeção estratégica de terceirização/EIS (queda para ~29k em 2035)
</commit_message>
<xml_diff>
--- a/dados/pessoal_tratado.xlsx
+++ b/dados/pessoal_tratado.xlsx
@@ -1363,22 +1363,22 @@
         <v>2026</v>
       </c>
       <c r="B2" t="n">
-        <v>495</v>
+        <v>500</v>
       </c>
       <c r="C2" t="n">
-        <v>880</v>
+        <v>900</v>
       </c>
       <c r="D2" t="n">
-        <v>330</v>
+        <v>350</v>
       </c>
       <c r="E2" t="n">
         <v>10100</v>
       </c>
       <c r="F2" t="n">
-        <v>11805</v>
+        <v>11850</v>
       </c>
       <c r="G2" t="n">
-        <v>76284</v>
+        <v>76239</v>
       </c>
     </row>
     <row r="3">
@@ -1386,22 +1386,22 @@
         <v>2027</v>
       </c>
       <c r="B3" t="n">
-        <v>528</v>
+        <v>520</v>
       </c>
       <c r="C3" t="n">
-        <v>935</v>
+        <v>950</v>
       </c>
       <c r="D3" t="n">
-        <v>352</v>
+        <v>370</v>
       </c>
       <c r="E3" t="n">
         <v>3000</v>
       </c>
       <c r="F3" t="n">
-        <v>4815</v>
+        <v>4840</v>
       </c>
       <c r="G3" t="n">
-        <v>71469</v>
+        <v>71399</v>
       </c>
     </row>
     <row r="4">
@@ -1409,22 +1409,22 @@
         <v>2028</v>
       </c>
       <c r="B4" t="n">
-        <v>572</v>
+        <v>540</v>
       </c>
       <c r="C4" t="n">
-        <v>1013</v>
+        <v>1000</v>
       </c>
       <c r="D4" t="n">
-        <v>385</v>
+        <v>390</v>
       </c>
       <c r="E4" t="n">
         <v>3000</v>
       </c>
       <c r="F4" t="n">
-        <v>4970</v>
+        <v>4930</v>
       </c>
       <c r="G4" t="n">
-        <v>66499</v>
+        <v>66469</v>
       </c>
     </row>
     <row r="5">
@@ -1432,22 +1432,22 @@
         <v>2029</v>
       </c>
       <c r="B5" t="n">
-        <v>550</v>
+        <v>560</v>
       </c>
       <c r="C5" t="n">
-        <v>1090</v>
+        <v>1050</v>
       </c>
       <c r="D5" t="n">
-        <v>418</v>
+        <v>410</v>
       </c>
       <c r="E5" t="n">
         <v>3000</v>
       </c>
       <c r="F5" t="n">
-        <v>5058</v>
+        <v>5020</v>
       </c>
       <c r="G5" t="n">
-        <v>61441</v>
+        <v>61449</v>
       </c>
     </row>
     <row r="6">
@@ -1455,22 +1455,22 @@
         <v>2030</v>
       </c>
       <c r="B6" t="n">
-        <v>605</v>
+        <v>580</v>
       </c>
       <c r="C6" t="n">
-        <v>1156</v>
+        <v>1100</v>
       </c>
       <c r="D6" t="n">
-        <v>440</v>
+        <v>430</v>
       </c>
       <c r="E6" t="n">
         <v>3000</v>
       </c>
       <c r="F6" t="n">
-        <v>5201</v>
+        <v>5110</v>
       </c>
       <c r="G6" t="n">
-        <v>56240</v>
+        <v>56339</v>
       </c>
     </row>
     <row r="7">
@@ -1478,22 +1478,22 @@
         <v>2031</v>
       </c>
       <c r="B7" t="n">
-        <v>583</v>
+        <v>600</v>
       </c>
       <c r="C7" t="n">
-        <v>1211</v>
+        <v>1150</v>
       </c>
       <c r="D7" t="n">
-        <v>462</v>
+        <v>450</v>
       </c>
       <c r="E7" t="n">
         <v>3000</v>
       </c>
       <c r="F7" t="n">
-        <v>5256</v>
+        <v>5200</v>
       </c>
       <c r="G7" t="n">
-        <v>50984</v>
+        <v>51139</v>
       </c>
     </row>
     <row r="8">
@@ -1501,22 +1501,22 @@
         <v>2032</v>
       </c>
       <c r="B8" t="n">
-        <v>539</v>
+        <v>620</v>
       </c>
       <c r="C8" t="n">
-        <v>1266</v>
+        <v>1200</v>
       </c>
       <c r="D8" t="n">
-        <v>495</v>
+        <v>470</v>
       </c>
       <c r="E8" t="n">
         <v>3000</v>
       </c>
       <c r="F8" t="n">
-        <v>5300</v>
+        <v>5290</v>
       </c>
       <c r="G8" t="n">
-        <v>45684</v>
+        <v>45849</v>
       </c>
     </row>
     <row r="9">
@@ -1524,22 +1524,22 @@
         <v>2033</v>
       </c>
       <c r="B9" t="n">
-        <v>506</v>
+        <v>640</v>
       </c>
       <c r="C9" t="n">
-        <v>1321</v>
+        <v>1250</v>
       </c>
       <c r="D9" t="n">
-        <v>517</v>
+        <v>490</v>
       </c>
       <c r="E9" t="n">
         <v>3000</v>
       </c>
       <c r="F9" t="n">
-        <v>5344</v>
+        <v>5380</v>
       </c>
       <c r="G9" t="n">
-        <v>40340</v>
+        <v>40469</v>
       </c>
     </row>
     <row r="10">
@@ -1547,22 +1547,22 @@
         <v>2034</v>
       </c>
       <c r="B10" t="n">
-        <v>473</v>
+        <v>660</v>
       </c>
       <c r="C10" t="n">
-        <v>1299</v>
+        <v>1300</v>
       </c>
       <c r="D10" t="n">
-        <v>539</v>
+        <v>510</v>
       </c>
       <c r="E10" t="n">
         <v>3000</v>
       </c>
       <c r="F10" t="n">
-        <v>5311</v>
+        <v>5470</v>
       </c>
       <c r="G10" t="n">
-        <v>35029</v>
+        <v>34999</v>
       </c>
     </row>
     <row r="11">
@@ -1570,22 +1570,22 @@
         <v>2035</v>
       </c>
       <c r="B11" t="n">
-        <v>451</v>
+        <v>680</v>
       </c>
       <c r="C11" t="n">
-        <v>1211</v>
+        <v>1350</v>
       </c>
       <c r="D11" t="n">
-        <v>550</v>
+        <v>530</v>
       </c>
       <c r="E11" t="n">
         <v>3000</v>
       </c>
       <c r="F11" t="n">
-        <v>5212</v>
+        <v>5560</v>
       </c>
       <c r="G11" t="n">
-        <v>29817</v>
+        <v>29439</v>
       </c>
     </row>
   </sheetData>

</xml_diff>